<commit_message>
2026-05-09 update: backtest period 2000-2010, reward function v3, walk-forward v2, safe PPO
</commit_message>
<xml_diff>
--- a/taiwan_stock_.xlsx
+++ b/taiwan_stock_.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\Isaac_WORK\private\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8593E5A-E2AC-46FB-9098-8849D8CE993A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09222B9C-E72B-4E5F-B8CA-E805EFC619C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CB0707DF-3E0B-4A32-9B95-35D7B926E757}"/>
   </bookViews>
@@ -24,44 +24,53 @@
   <si>
     <t>元大台灣50 
 0050</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
     <t>元大高股息
 0056</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
     <t>元大S&amp;P500 
 00646</t>
+    <phoneticPr fontId="21" type="noConversion"/>
   </si>
   <si>
     <t>元大美債20年
 00679B</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
     <t>元大台灣高息低波
 00713</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
     <t>元大AAA至A公司債
 00751B</t>
+    <phoneticPr fontId="21" type="noConversion"/>
   </si>
   <si>
     <t>國泰永續高股息
 00878</t>
+    <phoneticPr fontId="20" type="noConversion"/>
+  </si>
+  <si>
+    <t>即時庫存</t>
+    <phoneticPr fontId="21" type="noConversion"/>
   </si>
   <si>
     <t>玉山金
 2884</t>
-  </si>
-  <si>
-    <t>即時庫存</t>
+    <phoneticPr fontId="20" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -220,6 +229,25 @@
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="33">
@@ -519,7 +547,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
@@ -646,16 +674,22 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="42" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - 輔色1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - 輔色2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - 輔色3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -675,6 +709,7 @@
     <cellStyle name="60% - 輔色5" xfId="37" builtinId="48" customBuiltin="1"/>
     <cellStyle name="60% - 輔色6" xfId="41" builtinId="52" customBuiltin="1"/>
     <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="一般 2" xfId="42" xr:uid="{892FC553-202D-4244-8A1E-C0F0025D0EF1}"/>
     <cellStyle name="中等" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="合計" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="好" xfId="6" builtinId="26" customBuiltin="1"/>
@@ -1010,43 +1045,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF61596-49CC-406B-88F6-E78A6874A4F3}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="17"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="68" x14ac:dyDescent="0.4">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:9" ht="68">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
       <c r="B2">
-        <v>1036</v>
+        <v>1089</v>
       </c>
       <c r="C2">
-        <v>16429</v>
+        <v>16673</v>
       </c>
       <c r="D2">
         <v>32</v>
@@ -1055,13 +1090,13 @@
         <v>23000</v>
       </c>
       <c r="F2">
-        <v>4686</v>
+        <v>4780</v>
       </c>
       <c r="G2">
         <v>1000</v>
       </c>
       <c r="H2">
-        <v>13836</v>
+        <v>14236</v>
       </c>
       <c r="I2">
         <v>20</v>

</xml_diff>